<commit_message>
Corrige parser Q10: verifica início da string em vez de substring
Bug: "COCRIADOR - ...construir o novo que precisa surgir" contém "novo",
causando parse errado (retornava Novo em vez de Cocriador).
Fix: usa startswith em vez de 'in' para match do nome do estágio.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaN6iQfVUePBZHakcrumrR
</commit_message>
<xml_diff>
--- a/classificacao_individual.xlsx
+++ b/classificacao_individual.xlsx
@@ -56,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009FC5E8"/>
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,7 +71,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="009FC5E8"/>
       </patternFill>
     </fill>
     <fill>
@@ -675,7 +675,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Potencial +2 ou mais níveis</t>
+          <t>Alinhado</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -926,12 +926,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1050,7 +1050,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -1174,12 +1174,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1298,12 +1298,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1422,12 +1422,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1546,12 +1546,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1675,7 +1675,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -1794,12 +1794,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -1918,7 +1918,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -2166,12 +2166,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -2295,7 +2295,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -2414,7 +2414,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -2543,7 +2543,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -2662,12 +2662,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -2786,7 +2786,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -3034,12 +3034,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -3158,7 +3158,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -3287,7 +3287,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -3411,7 +3411,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -3530,12 +3530,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -3783,9 +3783,9 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3902,12 +3902,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -4031,7 +4031,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -4150,7 +4150,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -4274,12 +4274,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -4398,12 +4398,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -4646,7 +4646,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -4767,17 +4767,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Novo</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
+          <t>Cocriador</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4899,7 +4899,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -5018,12 +5018,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -5139,7 +5139,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -5147,9 +5147,9 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -5271,7 +5271,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -5519,7 +5519,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -5643,9 +5643,9 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -5767,7 +5767,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -5886,12 +5886,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -6134,7 +6134,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -6258,7 +6258,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -6387,7 +6387,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6506,12 +6506,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6635,7 +6635,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6754,7 +6754,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -6878,12 +6878,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -7002,12 +7002,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -7126,7 +7126,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -7250,7 +7250,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -7374,7 +7374,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -7503,7 +7503,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -7746,7 +7746,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -7870,12 +7870,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -7994,7 +7994,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -8118,7 +8118,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -8371,7 +8371,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -8490,12 +8490,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -8614,12 +8614,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -8862,12 +8862,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G68" s="6" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -8986,12 +8986,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -9110,12 +9110,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr">
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -9234,12 +9234,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F71" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -9358,12 +9358,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F72" s="6" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G72" s="6" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -9482,12 +9482,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F73" s="6" t="inlineStr">
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G73" s="6" t="inlineStr">
+      <c r="G73" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -9606,12 +9606,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F74" s="6" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -9730,7 +9730,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F75" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -9854,12 +9854,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F76" s="6" t="inlineStr">
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G76" s="3" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -9978,12 +9978,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G77" s="6" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -10102,12 +10102,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F78" s="6" t="inlineStr">
+      <c r="F78" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G78" s="3" t="inlineStr">
+      <c r="G78" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10226,7 +10226,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F79" s="6" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -10474,7 +10474,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F81" s="6" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -10598,12 +10598,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F82" s="6" t="inlineStr">
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G82" s="3" t="inlineStr">
+      <c r="G82" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10722,12 +10722,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F83" s="6" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G83" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -10846,12 +10846,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F84" s="6" t="inlineStr">
+      <c r="F84" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G84" s="3" t="inlineStr">
+      <c r="G84" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10970,12 +10970,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F85" s="6" t="inlineStr">
+      <c r="F85" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G85" s="6" t="inlineStr">
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -11094,12 +11094,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -11223,7 +11223,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G87" s="3" t="inlineStr">
+      <c r="G87" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -11347,7 +11347,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G88" s="3" t="inlineStr">
+      <c r="G88" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -11471,9 +11471,9 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G89" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -11590,12 +11590,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
+      <c r="F90" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="G90" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -11714,12 +11714,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="F91" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -11959,17 +11959,17 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Novo</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr">
+          <t>Cocriador</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G93" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -12210,12 +12210,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F95" s="6" t="inlineStr">
+      <c r="F95" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G95" s="6" t="inlineStr">
+      <c r="G95" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -12331,17 +12331,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Novo</t>
-        </is>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
+          <t>Cocriador</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G96" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -12458,12 +12458,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F97" s="6" t="inlineStr">
+      <c r="F97" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G97" s="6" t="inlineStr">
+      <c r="G97" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -12582,12 +12582,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="F98" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G98" s="6" t="inlineStr">
+      <c r="G98" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -12706,7 +12706,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -12830,12 +12830,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F100" s="6" t="inlineStr">
+      <c r="F100" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G100" s="3" t="inlineStr">
+      <c r="G100" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -12959,7 +12959,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G101" s="3" t="inlineStr">
+      <c r="G101" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13078,12 +13078,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
+      <c r="F102" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G102" s="3" t="inlineStr">
+      <c r="G102" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13202,12 +13202,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F103" s="6" t="inlineStr">
+      <c r="F103" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G103" s="3" t="inlineStr">
+      <c r="G103" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13450,12 +13450,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F105" s="6" t="inlineStr">
+      <c r="F105" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G105" s="3" t="inlineStr">
+      <c r="G105" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13579,7 +13579,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G106" s="3" t="inlineStr">
+      <c r="G106" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13698,12 +13698,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F107" s="6" t="inlineStr">
+      <c r="F107" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G107" s="3" t="inlineStr">
+      <c r="G107" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13822,12 +13822,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F108" s="6" t="inlineStr">
+      <c r="F108" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G108" s="6" t="inlineStr">
+      <c r="G108" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -13946,12 +13946,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F109" s="6" t="inlineStr">
+      <c r="F109" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G109" s="3" t="inlineStr">
+      <c r="G109" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -14075,7 +14075,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G110" s="3" t="inlineStr">
+      <c r="G110" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -14318,7 +14318,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="F112" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -14442,12 +14442,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F113" s="6" t="inlineStr">
+      <c r="F113" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G113" s="3" t="inlineStr">
+      <c r="G113" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -14690,12 +14690,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F115" s="6" t="inlineStr">
+      <c r="F115" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G115" s="6" t="inlineStr">
+      <c r="G115" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -14814,7 +14814,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="F116" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -14938,12 +14938,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F117" s="6" t="inlineStr">
+      <c r="F117" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G117" s="6" t="inlineStr">
+      <c r="G117" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -15062,12 +15062,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F118" s="6" t="inlineStr">
+      <c r="F118" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G118" s="6" t="inlineStr">
+      <c r="G118" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -15191,7 +15191,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G119" s="3" t="inlineStr">
+      <c r="G119" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -15310,12 +15310,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F120" s="6" t="inlineStr">
+      <c r="F120" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G120" s="6" t="inlineStr">
+      <c r="G120" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -15434,7 +15434,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F121" s="6" t="inlineStr">
+      <c r="F121" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -15558,12 +15558,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F122" s="6" t="inlineStr">
+      <c r="F122" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G122" s="3" t="inlineStr">
+      <c r="G122" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Novo</t>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="F123" s="7" t="inlineStr">
@@ -15687,9 +15687,9 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G123" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -15935,7 +15935,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="G125" s="6" t="inlineStr">
+      <c r="G125" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -16178,12 +16178,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F127" s="6" t="inlineStr">
+      <c r="F127" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G127" s="3" t="inlineStr">
+      <c r="G127" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -16302,7 +16302,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F128" s="6" t="inlineStr">
+      <c r="F128" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -16426,12 +16426,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F129" s="6" t="inlineStr">
+      <c r="F129" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G129" s="3" t="inlineStr">
+      <c r="G129" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -16547,17 +16547,17 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Novo</t>
-        </is>
-      </c>
-      <c r="F130" s="6" t="inlineStr">
+          <t>Cocriador</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G130" s="3" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -16674,12 +16674,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F131" s="6" t="inlineStr">
+      <c r="F131" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G131" s="3" t="inlineStr">
+      <c r="G131" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -16798,12 +16798,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F132" s="6" t="inlineStr">
+      <c r="F132" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G132" s="3" t="inlineStr">
+      <c r="G132" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -16922,7 +16922,7 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F133" s="6" t="inlineStr">
+      <c r="F133" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -17046,12 +17046,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F134" s="6" t="inlineStr">
+      <c r="F134" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G134" s="3" t="inlineStr">
+      <c r="G134" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17170,12 +17170,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F135" s="6" t="inlineStr">
+      <c r="F135" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G135" s="6" t="inlineStr">
+      <c r="G135" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
@@ -17294,12 +17294,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F136" s="6" t="inlineStr">
+      <c r="F136" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G136" s="3" t="inlineStr">
+      <c r="G136" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17418,12 +17418,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F137" s="6" t="inlineStr">
+      <c r="F137" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G137" s="3" t="inlineStr">
+      <c r="G137" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17542,12 +17542,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F138" s="6" t="inlineStr">
+      <c r="F138" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G138" s="3" t="inlineStr">
+      <c r="G138" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17666,7 +17666,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F139" s="6" t="inlineStr">
+      <c r="F139" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
@@ -17790,12 +17790,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F140" s="6" t="inlineStr">
+      <c r="F140" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G140" s="3" t="inlineStr">
+      <c r="G140" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17914,12 +17914,12 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F141" s="6" t="inlineStr">
+      <c r="F141" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G141" s="3" t="inlineStr">
+      <c r="G141" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18038,12 +18038,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F142" s="6" t="inlineStr">
+      <c r="F142" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G142" s="3" t="inlineStr">
+      <c r="G142" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18162,12 +18162,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F143" s="6" t="inlineStr">
+      <c r="F143" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G143" s="3" t="inlineStr">
+      <c r="G143" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18286,12 +18286,12 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F144" s="6" t="inlineStr">
+      <c r="F144" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G144" s="3" t="inlineStr">
+      <c r="G144" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18491,20 +18491,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>68.5%</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Disse SIM, mas ainda sem papel ativo estruturado</t>
         </is>
@@ -18597,7 +18597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -18668,19 +18668,15 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -18799,29 +18795,54 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cocriador</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
         <v>98</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F9" t="n">
         <v>24</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G9" t="n">
         <v>11</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H9" t="n">
         <v>9</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I9" t="n">
         <v>143</v>
       </c>
     </row>
@@ -18868,17 +18889,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Alinhado</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>31.5%</t>
+          <t>32.2%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -18908,17 +18929,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>37.8%</t>
+          <t>30.8%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18934,11 +18955,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>12.6%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -18954,11 +18975,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona teto de estágio para novatos (≤1 ano na escola)
Pessoas que entraram em 2024 ou 2025 são capadas em Inserindo independente
do nível de concordância: a adaptação e absorção da escola requerem tempo
antes da decisão real de comprometimento. Alta concordância é registrada na
justificativa como "potencial para Comprometido" e reflete no próximo nível.

Resultado: 46 em Inserindo (38 de 2025 + parte de 2024),
Comprometido cai de 98 → 64.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaN6iQfVUePBZHakcrumrR
</commit_message>
<xml_diff>
--- a/classificacao_individual.xlsx
+++ b/classificacao_individual.xlsx
@@ -71,7 +71,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="009FC5E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA9999"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,17 +96,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EA9999"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1422,34 +1422,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1675,7 +1675,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -1918,34 +1918,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Autoposicionamento +1 acima</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2042,34 +2042,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Embaixador</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2 papéis ativos + concordância global (92%)</t>
+          <t>Alta concordância / engajamento (potencial Embaixador), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Cocriador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Engajar na co-criação: grupos estratégicos, mentoria, novos projetos</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Embaixador — referência e representante da escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2166,34 +2166,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2295,7 +2295,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -2786,34 +2786,34 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Alinhado</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=92%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2910,7 +2910,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -3282,34 +3282,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (77%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 0 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3411,7 +3411,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -3654,12 +3654,12 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -3778,7 +3778,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -4026,34 +4026,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (94%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 0 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -4150,34 +4150,34 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Alinhado</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -4646,34 +4646,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Autoposicionamento +1 acima</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -4775,7 +4775,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -4899,7 +4899,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -5018,34 +5018,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -5147,7 +5147,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G38" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -5266,34 +5266,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (93%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -5514,7 +5514,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -5638,34 +5638,34 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Embaixador</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Autoposicionamento +1 acima</t>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2 papéis ativos + concordância global (95%)</t>
+          <t>Alta concordância / engajamento (potencial Embaixador), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Cocriador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Engajar na co-criação: grupos estratégicos, mentoria, novos projetos</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Embaixador — referência e representante da escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -5767,7 +5767,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6010,34 +6010,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (95%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -6263,7 +6263,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G47" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -6387,7 +6387,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6506,34 +6506,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -6635,7 +6635,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -6878,34 +6878,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -7007,7 +7007,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -7503,7 +7503,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -7870,34 +7870,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=92%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -8123,7 +8123,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G62" s="9" t="inlineStr">
+      <c r="G62" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -8366,34 +8366,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (81%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -8614,34 +8614,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -8986,34 +8986,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F69" s="3" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -9859,7 +9859,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G76" s="6" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10107,7 +10107,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="G78" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10603,7 +10603,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="G82" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -10851,7 +10851,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G84" s="6" t="inlineStr">
+      <c r="G84" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -11218,34 +11218,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>Cocriador</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>3 papéis ativos + concordância global (95%) + Ec. Fraterna forte (100%)</t>
+          <t>Alta concordância / engajamento (potencial Cocriador), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Cocriador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Manter e ampliar a co-criação — já no topo da curva</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Cocriador — co-constrói o futuro da escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -11347,7 +11347,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="G88" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -11471,7 +11471,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G89" s="9" t="inlineStr">
+      <c r="G89" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -11967,7 +11967,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G93" s="9" t="inlineStr">
+      <c r="G93" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -12086,9 +12086,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F94" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
+      <c r="F94" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -12098,22 +12098,22 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (87%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 0 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -12210,34 +12210,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F95" s="3" t="inlineStr">
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G95" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -12339,7 +12339,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G96" s="9" t="inlineStr">
+      <c r="G96" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -12835,7 +12835,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G100" s="6" t="inlineStr">
+      <c r="G100" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -12959,7 +12959,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="G101" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -13078,34 +13078,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F102" s="3" t="inlineStr">
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G102" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G102" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -13202,34 +13202,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F103" s="3" t="inlineStr">
+      <c r="F103" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G103" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -13326,7 +13326,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F104" s="7" t="inlineStr">
+      <c r="F104" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -13450,34 +13450,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F105" s="3" t="inlineStr">
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=88%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G105" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -13574,34 +13574,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F106" s="7" t="inlineStr">
-        <is>
-          <t>Embaixador</t>
-        </is>
-      </c>
-      <c r="G106" s="6" t="inlineStr">
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2 papéis ativos + concordância global (71%)</t>
+          <t>Alta concordância / engajamento (potencial Embaixador), mas tempo na escola: 0 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Cocriador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>Engajar na co-criação: grupos estratégicos, mentoria, novos projetos</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Embaixador — referência e representante da escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -13698,34 +13698,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F107" s="3" t="inlineStr">
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G107" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -13946,34 +13946,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F109" s="3" t="inlineStr">
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G109" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -14075,7 +14075,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="G110" s="6" t="inlineStr">
+      <c r="G110" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -14447,7 +14447,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G113" s="6" t="inlineStr">
+      <c r="G113" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -14690,34 +14690,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F115" s="3" t="inlineStr">
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G115" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -14814,34 +14814,34 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F116" s="3" t="inlineStr">
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>Alinhado</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G116" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -14938,34 +14938,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F117" s="3" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G117" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -15186,34 +15186,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F119" s="4" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
-      <c r="G119" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1 papel(éis) ativo(s) + concordância (98%)</t>
+          <t>Alta concordância / engajamento (potencial Ativo no Motivo), mas tempo na escola: 0 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Embaixador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Ampliar atuação para 2+ papéis e fortalecer prática da Ec. Fraterna</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Colaborador ativo — tem papel definido na escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -15558,34 +15558,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F122" s="3" t="inlineStr">
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G122" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -15682,7 +15682,7 @@
           <t>Cocriador</t>
         </is>
       </c>
-      <c r="F123" s="7" t="inlineStr">
+      <c r="F123" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -15806,34 +15806,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F124" s="7" t="inlineStr">
-        <is>
-          <t>Embaixador</t>
-        </is>
-      </c>
-      <c r="G124" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G124" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>3 papéis ativos + concordância global (73%)</t>
+          <t>Alta concordância / engajamento (potencial Embaixador), mas tempo na escola: 1 ano(s) → cap em Inserindo</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Cocriador</t>
+          <t>Comprometido</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>Engajar na co-criação: grupos estratégicos, mentoria, novos projetos</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Embaixador — referência e representante da escola</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -15930,7 +15930,7 @@
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="F125" s="7" t="inlineStr">
+      <c r="F125" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -16054,7 +16054,7 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F126" s="7" t="inlineStr">
+      <c r="F126" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
@@ -16178,34 +16178,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F127" s="3" t="inlineStr">
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=92%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G127" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -16302,34 +16302,34 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F128" s="3" t="inlineStr">
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=92%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -16426,34 +16426,34 @@
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="F129" s="3" t="inlineStr">
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>Potencial +1 nível</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=92%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G129" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -16555,7 +16555,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G130" s="9" t="inlineStr">
+      <c r="G130" s="8" t="inlineStr">
         <is>
           <t>Autoposicionamento +2 ou mais acima</t>
         </is>
@@ -16674,34 +16674,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F131" s="3" t="inlineStr">
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G131" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -16798,34 +16798,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F132" s="3" t="inlineStr">
+      <c r="F132" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G132" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=79%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G132" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -16922,34 +16922,34 @@
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="F133" s="3" t="inlineStr">
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Alinhado</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 1 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G133" s="4" t="inlineStr">
-        <is>
-          <t>Potencial +1 nível</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -17051,7 +17051,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G134" s="6" t="inlineStr">
+      <c r="G134" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17170,34 +17170,34 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F135" s="3" t="inlineStr">
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +1 acima</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G135" s="3" t="inlineStr">
-        <is>
-          <t>Alinhado</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -17294,34 +17294,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F136" s="3" t="inlineStr">
+      <c r="F136" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G136" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G136" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -17423,7 +17423,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G137" s="6" t="inlineStr">
+      <c r="G137" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -17542,34 +17542,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F138" s="3" t="inlineStr">
+      <c r="F138" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G138" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G138" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -17666,34 +17666,34 @@
           <t>Ativo no Motivo</t>
         </is>
       </c>
-      <c r="F139" s="3" t="inlineStr">
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G139" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=96%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G139" s="5" t="inlineStr">
-        <is>
-          <t>Autoposicionamento +1 acima</t>
-        </is>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -17790,34 +17790,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F140" s="3" t="inlineStr">
+      <c r="F140" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G140" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=100%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G140" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -17919,7 +17919,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G141" s="6" t="inlineStr">
+      <c r="G141" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18043,7 +18043,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G142" s="6" t="inlineStr">
+      <c r="G142" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18162,34 +18162,34 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="F143" s="3" t="inlineStr">
+      <c r="F143" s="6" t="inlineStr">
+        <is>
+          <t>Inserindo</t>
+        </is>
+      </c>
+      <c r="G143" s="7" t="inlineStr">
+        <is>
+          <t>Potencial +2 ou mais níveis</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Alta concordância (Pertencimento net=83%), mas tempo na escola: 0 ano(s) → Inserindo (potencial rápido para Comprometido)</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G143" s="6" t="inlineStr">
-        <is>
-          <t>Potencial +2 ou mais níveis</t>
-        </is>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>Diz SIM para a escola, mas sem papel ativo no momento</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>Ativo no Motivo</t>
-        </is>
-      </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Assumir um papel ativo (representante, voluntário, APG ou GT)</t>
+          <t>Decidir: dizer SIM para a Arandu e engajar como Comprometido</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Membro comprometido — escolheu a Arandu</t>
+          <t>Explorador — processando dúvidas, próximo à decisão</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -18291,7 +18291,7 @@
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="G144" s="6" t="inlineStr">
+      <c r="G144" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
@@ -18431,60 +18431,60 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Novo</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Ainda em reconhecimento — não internalizou propósito/missão</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>0.7%</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Assimilando como a escola funciona — pode ter tensões ou ser recente</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="B4" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>32.2%</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>No ponto de virada — precisa decidir SIM ou NÃO</t>
         </is>
@@ -18497,11 +18497,11 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>44.8%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -18517,11 +18517,11 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -18531,20 +18531,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>7.7%</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>4.9%</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>2+ papéis ativos + alta concordância — referência comunitária</t>
         </is>
@@ -18557,11 +18557,11 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -18666,14 +18666,14 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>14</v>
+      </c>
       <c r="E2" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>20</v>
@@ -18687,12 +18687,14 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -18708,9 +18710,11 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -18731,16 +18735,18 @@
       <c r="C5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
       <c r="E5" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>51</v>
@@ -18754,15 +18760,17 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
         <v>6</v>
@@ -18802,7 +18810,9 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" t="n">
         <v>4</v>
       </c>
@@ -18810,7 +18820,7 @@
         <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
@@ -18829,18 +18839,20 @@
       <c r="C9" t="n">
         <v>1</v>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>46</v>
+      </c>
       <c r="E9" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G9" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I9" t="n">
         <v>143</v>
@@ -18895,11 +18907,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -18915,11 +18927,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18929,17 +18941,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Potencial +2 ou mais níveis</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>30.8%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18955,31 +18967,31 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>17.5%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Declara 1 nível acima do que as respostas sustentam</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Autoposicionamento +2 ou mais acima</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>18</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>12.6%</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Declara 1 nível acima do que as respostas sustentam</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Autoposicionamento +2 ou mais acima</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>6.3%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -19035,7 +19047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -19113,274 +19125,286 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>≥ 5 anos + não disse SIM + disc. ≥ 25%</t>
+          <t>≤ 1 ano na escola (2024–2025)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>→ Adaptando (tensão/sinal de possível saída)</t>
+          <t>→ Cap máximo = Inserindo, mesmo com alta concordância (potencial indica próximo passo)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>≥ 5 anos + não disse SIM + disc. ≥ 25%</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>→ Adaptando (tensão/sinal de possível saída)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>≥ 5 anos + não disse SIM</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>→ Inserindo (no ponto de virada há muito tempo)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LADO ESQUERDO — não disse SIM</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Discordância Pertencimento ≥ 40%</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>→ Novo (resistência)</t>
-        </is>
-      </c>
+          <t>LADO ESQUERDO — não disse SIM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Não sei Pertencimento ≥ 50%</t>
+          <t>Discordância Pertencimento ≥ 40%</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>→ Novo (não reconhece a escola ainda)</t>
+          <t>→ Novo (resistência)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Conhecimento ≥ 75% + positivo Pertencimento ≥ 50%</t>
+          <t>Não sei Pertencimento ≥ 50%</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>→ Inserindo</t>
+          <t>→ Novo (não reconhece a escola ainda)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Conhecimento ≥ 50% ou positivo Pertencimento ≥ 35%</t>
+          <t>Conhecimento ≥ 75% + positivo Pertencimento ≥ 50%</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>→ Adaptando</t>
+          <t>→ Inserindo</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Conhecimento ≥ 50% ou positivo Pertencimento ≥ 35%</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>→ Adaptando</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Demais casos</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>→ Novo</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>LADO DIREITO — disse SIM</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Discordância Acordos ≥ 25% E Ec.Fraterna ≥ 25%</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>→ Comprometido (tensões práticas)</t>
-        </is>
-      </c>
+          <t>LADO DIREITO — disse SIM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Discordância Acordos ≥ 25%</t>
+          <t>Discordância Acordos ≥ 25% E Ec.Fraterna ≥ 25%</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>→ Comprometido (tensão nos acordos)</t>
+          <t>→ Comprometido (tensões práticas)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Discordância Ec. Fraterna ≥ 25%</t>
+          <t>Discordância Acordos ≥ 25%</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>→ Comprometido (tensão econômica)</t>
+          <t>→ Comprometido (tensão nos acordos)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Não sei Acordos ≥ 40% E Não sei EF ≥ 40%</t>
+          <t>Discordância Ec. Fraterna ≥ 25%</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>→ Comprometido (ainda aprendendo práticas)</t>
+          <t>→ Comprometido (tensão econômica)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sem papel ativo</t>
+          <t>Não sei Acordos ≥ 40% E Não sei EF ≥ 40%</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>→ Comprometido</t>
+          <t>→ Comprometido (ainda aprendendo práticas)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3+ papéis ativos + overall ≥ 75% + EF ≥ 60%</t>
+          <t>Sem papel ativo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>→ Cocriador</t>
+          <t>→ Comprometido</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2+ papéis ativos + overall ≥ 70%</t>
+          <t>3+ papéis ativos + overall ≥ 75% + EF ≥ 60%</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>→ Embaixador</t>
+          <t>→ Cocriador</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1+ papel ativo + overall ≥ 60%</t>
+          <t>2+ papéis ativos + overall ≥ 70%</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>→ Ativo no Motivo</t>
+          <t>→ Embaixador</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>1+ papel ativo + overall ≥ 60%</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>→ Ativo no Motivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Papel ativo + overall &lt; 60%</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>→ Comprometido</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>NET SIGNAL — exemplos</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Todos Concordo</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>net = (1,0+0,8)/1,8 = 1,00</t>
-        </is>
-      </c>
+          <t>NET SIGNAL — exemplos</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Todos Concordo parcialmente</t>
+          <t>Todos Concordo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>net = (0,4+0,8)/1,8 = 0,67</t>
+          <t>net = (1,0+0,8)/1,8 = 1,00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Todos Não sei opinar</t>
+          <t>Todos Concordo parcialmente</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>net = (−0,2+0,8)/1,8 = 0,33</t>
+          <t>net = (0,4+0,8)/1,8 = 0,67</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Todos Não sei opinar</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>net = (−0,2+0,8)/1,8 = 0,33</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Todos Discordo</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>net = (−0,8+0,8)/1,8 = 0,00</t>
         </is>

</xml_diff>